<commit_message>
Release 0.1.0: remove list-columns from datasets
washdev and uncnewsletter stored supp_file_type, supp_url,
das_repo_url, and keywords as list-columns, which broke flat-file
exports such as write.csv(). Collapse them into "; "-delimited
character columns in both datasets, update the data dictionary,
documentation, and the data availability article, and regenerate
the extdata exports, README, and pkgdown site.

Document the changes in NEWS.md, bump the version to 0.1.0, and
add alt text to the README word cloud figure.

Closes #8

Assisted-by: Claude claude-fable-5
</commit_message>
<xml_diff>
--- a/inst/extdata/uncnewsletter.xlsx
+++ b/inst/extdata/uncnewsletter.xlsx
@@ -131,7 +131,7 @@
     <t xml:space="preserve">0000-0002-5778-354X</t>
   </si>
   <si>
-    <t xml:space="preserve">c("drinkingwater", "environmentalpolicy", "healthandsafety")</t>
+    <t xml:space="preserve">drinkingwater; environmentalpolicy; healthandsafety</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/ieh0rf</t>
@@ -242,7 +242,7 @@
     <t xml:space="preserve">geekd@longwood.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Containerbreeding", "Mosquito", "Mosquitolarvae", "Rainwaterharvesting")</t>
+    <t xml:space="preserve">Containerbreeding; Mosquito; Mosquitolarvae; Rainwaterharvesting</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/icBZuL</t>
@@ -272,10 +272,10 @@
     <t xml:space="preserve">Cape Fear River Basin (eight-digit Hydrologic Unit Code 03030002) data sets utilized for this research are as follows: NCDMS Tier 1 project sites implemented prior to December 2015 (Division of Mitigation Services, 2019) available from the North Carolina Department of Environmental Quality at https://deq.nc.gov/about/divisions/mitigation-services/dms-planning/dms-web-map; parcel data (NC OneMap Geospatial Portal, 2019) available from NC OneMap at https://www.nconemap.gov/; land-use/land-cover data (Dewitz, 2019) available from the USGS ScienceBase at https://doi.org/10.5066/P96HHBIE; total phosphorus loads (Gurley et al., 2019) available from the USGS ScienceBase at https://doi.org/10.5066/P9UUT74V; hydric soils (Soil Survey Staff, 2019) available from the USDA Natural Resources Conservation Service at https://websoilsurvey.nrcs.usda.gov/; future development probability (Sanchez et al., 2020b) available from the USGS ScienceBase at https://doi.org/10.5066/P95PTP5G.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://deq.nc.gov/about/divisions/mitigation-services/dms-planning/dms-web-map", "https://www.nconemap.gov/", "https://doi.org/10.5066/P96HHBIE", "https://doi.org/10.5066/P9UUT74V", "https://websoilsurvey.nrcs.usda.gov/", "https://doi.org/10.5066/P95PTP5G")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("compensatorymitigation", "decisionscience", "knowledgecoproduction", "naturalresourcesmanagement", "research-managementpartnerships", "watershedplanning")</t>
+    <t xml:space="preserve">https://deq.nc.gov/about/divisions/mitigation-services/dms-planning/dms-web-map; https://www.nconemap.gov/; https://doi.org/10.5066/P96HHBIE; https://doi.org/10.5066/P9UUT74V; https://websoilsurvey.nrcs.usda.gov/; https://doi.org/10.5066/P95PTP5G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compensatorymitigation; decisionscience; knowledgecoproduction; naturalresourcesmanagement; research-managementpartnerships; watershedplanning</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/itNRLc</t>
@@ -302,7 +302,7 @@
     <t xml:space="preserve">lackstro@mailbox.sc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Drought", "Communications/decision-making", "Decisionsupport", "Localeffects", "Societalimpacts", "Community")</t>
+    <t xml:space="preserve">Drought; Communications/decision-making; Decisionsupport; Localeffects; Societalimpacts; Community</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/h4G3CX</t>
@@ -350,7 +350,7 @@
     <t xml:space="preserve">https://doi.org/10.15139/S3/BDQG9O</t>
   </si>
   <si>
-    <t xml:space="preserve">c("environmentaljustice", "privatewells", "toxicmetals")</t>
+    <t xml:space="preserve">environmentaljustice; privatewells; toxicmetals</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/im-ZMI</t>
@@ -383,7 +383,7 @@
     <t xml:space="preserve">on request</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Escherichiacoli", "Plasmid-mediatedquinoloneresistance", "Plasmid-mediatedcolistinresistance", "Poultryworkers", "Chicken", "PoultryEnvironments", "Nigeria")</t>
+    <t xml:space="preserve">Escherichiacoli; Plasmid-mediatedquinoloneresistance; Plasmid-mediatedcolistinresistance; Poultryworkers; Chicken; PoultryEnvironments; Nigeria</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/hZ8bR1</t>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">0000-0002-0371-7125</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Stakeholderanalysis", "FEWS", "Environmentalsustainability", "Transdisciplinaryresearch", "Stakeholderengagement", "Livestockproduction")</t>
+    <t xml:space="preserve">Stakeholderanalysis; FEWS; Environmentalsustainability; Transdisciplinaryresearch; Stakeholderengagement; Livestockproduction</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/iadi9z</t>
@@ -491,7 +491,7 @@
     <t xml:space="preserve">0000-0003-1591-3622</t>
   </si>
   <si>
-    <t xml:space="preserve">c("WaterResources", "Life", "EnvironmentalEducation", "Development", "UN2030Agenda")</t>
+    <t xml:space="preserve">WaterResources; Life; EnvironmentalEducation; Development; UN2030Agenda</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/irTmaA</t>
@@ -518,7 +518,7 @@
     <t xml:space="preserve">claire.mullaney@duke.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("water", "safedrinkingwateract", "environmentallaw", "law", "policy", "publichealth", "NorthCarolina")</t>
+    <t xml:space="preserve">water; safedrinkingwateract; environmentallaw; law; policy; publichealth; NorthCarolina</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/ipmsMg</t>
@@ -572,7 +572,7 @@
     <t xml:space="preserve">ekoso@smcm.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Algalblooms", "dynamicalsystems", "mathmodelling", "nutrienttresholdforresolvableblooms")</t>
+    <t xml:space="preserve">Algalblooms; dynamicalsystems; mathmodelling; nutrienttresholdforresolvableblooms</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.ajog.org/article/S0002-9378(22)01567-8/fulltext</t>
@@ -602,7 +602,7 @@
     <t xml:space="preserve">Blood concentrations of per- and polyfluoroalkyl substances are associated with autoimmune-like effects in American alligators from Wilmington, North Carolina</t>
   </si>
   <si>
-    <t xml:space="preserve">c("xlsx", "docx")</t>
+    <t xml:space="preserve">xlsx; docx</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.frontiersin.org/articles/10.3389/ftox.2022.1010185/full#supplementary-material</t>
@@ -623,7 +623,7 @@
     <t xml:space="preserve">The datasets presented in this study can be found in online repositories. The names of the repository/repositories and accession number(s) can be found in the article/Supplementary Material.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("autoantibodies", "autoimmune", "crocodilian", "immunetoxicity", "lupus", "onehealth")</t>
+    <t xml:space="preserve">autoantibodies; autoimmune; crocodilian; immunetoxicity; lupus; onehealth</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/h7S0S1</t>
@@ -692,7 +692,7 @@
     <t xml:space="preserve">0000-0002-5347-1370</t>
   </si>
   <si>
-    <t xml:space="preserve">c("privatewells", "environmentaljustice", "drinkingwater", "testing", "metalcontamination")</t>
+    <t xml:space="preserve">privatewells; environmentaljustice; drinkingwater; testing; metalcontamination</t>
   </si>
   <si>
     <t xml:space="preserve">https://ascelibrary.org/doi/abs/10.1061/JWRMD5.WRENG-5863</t>
@@ -767,7 +767,7 @@
     <t xml:space="preserve">catherine.otero@duke.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Infrastructure", "NorthCarolina", "Hurricanes", "NaturalDisasters", "PublicOpinion", "WaterSystems")</t>
+    <t xml:space="preserve">Infrastructure; NorthCarolina; Hurricanes; NaturalDisasters; PublicOpinion; WaterSystems</t>
   </si>
   <si>
     <t xml:space="preserve">https://awwa.onlinelibrary.wiley.com/doi/abs/10.1002/awwa.1977</t>
@@ -782,7 +782,7 @@
     <t xml:space="preserve">ahthomp4@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Utilities", "FinancialAssistance", "Durham", "NorthCarolina")</t>
+    <t xml:space="preserve">Utilities; FinancialAssistance; Durham; NorthCarolina</t>
   </si>
   <si>
     <t xml:space="preserve">https://journals.lww.com/environepidem/Fulltext/2022/08000/Associations_between_PFAS_occurrence_and.3.aspx?context=LatestArticles</t>
@@ -812,7 +812,7 @@
     <t xml:space="preserve">0000-0002-6322-4349</t>
   </si>
   <si>
-    <t xml:space="preserve">c("PFAS", "Multimorbidity", "ElectronicHealthRecords", "PFOA", "PFHpA", "Chronicdisease")</t>
+    <t xml:space="preserve">PFAS; Multimorbidity; ElectronicHealthRecords; PFOA; PFHpA; Chronicdisease</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/h2UiZf</t>
@@ -839,7 +839,7 @@
     <t xml:space="preserve">0000-0001-7584-8856</t>
   </si>
   <si>
-    <t xml:space="preserve">c("DrinkingWater", "Nitrate", "Disinfectionbyproducts", "Trihalomethanes", "Exposureassessment", "Agriculture", "Cohort")</t>
+    <t xml:space="preserve">DrinkingWater; Nitrate; Disinfectionbyproducts; Trihalomethanes; Exposureassessment; Agriculture; Cohort</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/h9U0Mr</t>
@@ -926,7 +926,7 @@
     <t xml:space="preserve">Effectiveness of interventions to improve drinking water, sanitation, and handwashing with soap on risk of diarrhoeal disease in children in low-income and middle-income settings: a systematic review and meta-analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">c("pdf", "xlsx")</t>
+    <t xml:space="preserve">pdf; xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">https://ars.els-cdn.com/content/image/1-s2.0-S0140673622009370-mmc1.xlsx</t>
@@ -956,7 +956,7 @@
     <t xml:space="preserve">Using detrending to assess SARS-CoV-2 wastewater loads as a leading indicator of fluctuations in COVID-19 cases at fine temporal scales: Correlations across twenty sewersheds in North Carolina</t>
   </si>
   <si>
-    <t xml:space="preserve">c("pdf", "code")</t>
+    <t xml:space="preserve">pdf; code</t>
   </si>
   <si>
     <t xml:space="preserve">Kelly Hoffman</t>
@@ -977,7 +977,7 @@
     <t xml:space="preserve">0000-0003-3925-1475</t>
   </si>
   <si>
-    <t xml:space="preserve">c("COVID19", "Viralload", "SARSCoV2", "Epidemiology", "Publicandoccupationalhealth", "NorthCarolina", "Diseasesurveillance", "Virustesting")</t>
+    <t xml:space="preserve">COVID19; Viralload; SARSCoV2; Epidemiology; Publicandoccupationalhealth; NorthCarolina; Diseasesurveillance; Virustesting</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/hXG2ID</t>
@@ -1082,7 +1082,7 @@
     <t xml:space="preserve">The data is available upon request. Please contact the corresponding author.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("TropicalCyclones", "Spectralwavemodelling", "Coastalhydrodynamics", "Oceancurrents", "Stormsurge", "Barrierislands")</t>
+    <t xml:space="preserve">TropicalCyclones; Spectralwavemodelling; Coastalhydrodynamics; Oceancurrents; Stormsurge; Barrierislands</t>
   </si>
   <si>
     <t xml:space="preserve">https://link.springer.com/article/10.1007/s13157-022-01605-y</t>
@@ -1112,7 +1112,7 @@
     <t xml:space="preserve">The datasets generated during and analyzed during the current study are available from the corresponding author on reasonable request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Pocosin", "Greenhousegases", "Restoration", "Mitigation")</t>
+    <t xml:space="preserve">Pocosin; Greenhousegases; Restoration; Mitigation</t>
   </si>
   <si>
     <t xml:space="preserve">https://link.springer.com/article/10.1007/s10980-022-01425-9</t>
@@ -1136,10 +1136,10 @@
     <t xml:space="preserve">All data used in this study was publicly available online. Eddy covariance data was downloaded from Ameriflux (https://ameriflux.lbl.gov/sites/siteinfo/US-Cwt). GRIDMET SPI data, land cover data, and USGS NED data was downloaded from Google Earth Engine (https://earthengine.google.com/). MODIS ET data was downloaded from USGS (https://lpdaac.usgs.gov/products/mod16a2gfv006/). Landsat ET data was downloaded from USGS (https://www.usgs.gov/core-science-systems/nli/landsat/landsat-provisional-actual-evapotranspiration). The Riley et al. (2021) forest composition map was downloaded from the USDA Forest Service (https://www.fs.usda.gov/rds/archive/Catalog/RDS-2019-0026). The Wilson et al. (2013) forest composition maps were downloaded from the USDA forest service (https://www.fs.usda.gov/rds/archive/catalog/RDS-2013-0013).</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://ameriflux.lbl.gov/sites/siteinfo/US-Cwt", "https://earthengine.google.com", "https://lpdaac.usgs.gov/products/mod16a2gfv006", "https://www.usgs.gov/core-science-systems/nli/landsat/landsat-provisional-actual-evapotranspiration", "https://www.fs.usda.gov/rds/archive/Catalog/RDS-2019-0026", "https://www.fs.usda.gov/rds/archive/catalog/RDS-2013-0013")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Evapotranspiration", "Remotesensing", "Topography", "Forestcomposition", "Landsat", "MODIS")</t>
+    <t xml:space="preserve">https://ameriflux.lbl.gov/sites/siteinfo/US-Cwt; https://earthengine.google.com; https://lpdaac.usgs.gov/products/mod16a2gfv006; https://www.usgs.gov/core-science-systems/nli/landsat/landsat-provisional-actual-evapotranspiration; https://www.fs.usda.gov/rds/archive/Catalog/RDS-2019-0026; https://www.fs.usda.gov/rds/archive/catalog/RDS-2013-0013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evapotranspiration; Remotesensing; Topography; Forestcomposition; Landsat; MODIS</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.pnas.org/doi/10.1073/pnas.2216021120</t>
@@ -1172,10 +1172,10 @@
     <t xml:space="preserve">Data (calculator and programming code) have been deposited in Covid-SURGE toolkit (21). Anonymized wastewater and case count data have been deposited in NC COVID dashboard (20). Some study data are available. The use of the Covid-SURGE algorithm or calculator beyond the scope of the CC BY-NC-ND 2.0 license is subject to permission being granted by Mathematica.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://wastewater.covidsurge.mathematica.org", "https://covid19.ncdhhs.gov/dashboard/data-behind-dashboards")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("WastewaterMonitoring", "Sars-Covid-2", "Covid-19Surge", "EarlyWarning", "AlertAlgorithm")</t>
+    <t xml:space="preserve">https://wastewater.covidsurge.mathematica.org; https://covid19.ncdhhs.gov/dashboard/data-behind-dashboards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WastewaterMonitoring; Sars-Covid-2; Covid-19Surge; EarlyWarning; AlertAlgorithm</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.pnas.org/doi/abs/10.1073/pnas.2120252120</t>
@@ -1205,7 +1205,7 @@
     <t xml:space="preserve">https://doi.org/10.7910/DVN/XT3RZ8</t>
   </si>
   <si>
-    <t xml:space="preserve">c("NonmarketEvaluation", "Waterquality", "Urbanstreams", "Statedpreference")</t>
+    <t xml:space="preserve">NonmarketEvaluation; Waterquality; Urbanstreams; Statedpreference</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.pnas.org/content/119/6/e2110694119.short</t>
@@ -1232,10 +1232,10 @@
     <t xml:space="preserve">Anonymized de-identified children's blood Pb, water source, household information, census block group information, and juvenile justice report data have been deposited in https://scholarworks.iu.edu/dspace/handle/2022/27027 (72, 73). https://scholarworks.iu.edu/dspace/handle/2022/25638.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://scholarworks.iu.edu/dspace/handle/2022/27027", "https://scholarworks.iu.edu/dspace/handle/2022/25638")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Drinkingwater", "Children", "Leadexposure")</t>
+    <t xml:space="preserve">https://scholarworks.iu.edu/dspace/handle/2022/27027; https://scholarworks.iu.edu/dspace/handle/2022/25638</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drinkingwater; Children; Leadexposure</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.tandfonline.com/doi/abs/10.1080/21622515.2023.2182719</t>
@@ -1259,7 +1259,7 @@
     <t xml:space="preserve">0000-0002-3317-7318</t>
   </si>
   <si>
-    <t xml:space="preserve">c("FaecalSludgeTreatment", "Composting", "Temperature-timecritera", "pathogeninactivationmechanism", "compostsanitation")</t>
+    <t xml:space="preserve">FaecalSludgeTreatment; Composting; Temperature-timecritera; pathogeninactivationmechanism; compostsanitation</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.tandfonline.com/doi/full/10.1080/09640568.2023.2183112</t>
@@ -1286,7 +1286,7 @@
     <t xml:space="preserve">0000-0003-2315-7062</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Hazardmitigation", "compoundevent", "flooding", "ruralresilience", "climatechange")</t>
+    <t xml:space="preserve">Hazardmitigation; compoundevent; flooding; ruralresilience; climatechange</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.tandfonline.com/doi/abs/10.1080/02626667.2022.2052073</t>
@@ -1310,7 +1310,7 @@
     <t xml:space="preserve">0000-0003-3160-5363</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Environmentaljustive", "Ambientwaterquality", "Interfaceswithsociety")</t>
+    <t xml:space="preserve">Environmentaljustive; Ambientwaterquality; Interfaceswithsociety</t>
   </si>
   <si>
     <t xml:space="preserve">https://agupubs.onlinelibrary.wiley.com/doi/full/10.1029/2021WR031533</t>
@@ -1343,7 +1343,7 @@
     <t xml:space="preserve">https://www.hydroshare.org/resource/b9fb89d2539c4e43b51889770f7a81f7</t>
   </si>
   <si>
-    <t xml:space="preserve">c("urban", "nonpointsource", "watershed", "nitrogen", "hydrology", "management")</t>
+    <t xml:space="preserve">urban; nonpointsource; watershed; nitrogen; hydrology; management</t>
   </si>
   <si>
     <t xml:space="preserve">https://agupubs.onlinelibrary.wiley.com/doi/full/10.1029/2021WR030711</t>
@@ -1376,7 +1376,7 @@
     <t xml:space="preserve">https://doi.org/10.4211/hs.c169de42e6174baf842a319efe28a75e</t>
   </si>
   <si>
-    <t xml:space="preserve">c("sandhills", "seepageflux", "groundwater", "surfacewater", "spatialvariability", "hydrology")</t>
+    <t xml:space="preserve">sandhills; seepageflux; groundwater; surfacewater; spatialvariability; hydrology</t>
   </si>
   <si>
     <t xml:space="preserve">https://agupubs.onlinelibrary.wiley.com/doi/10.1029/2021WR030700</t>
@@ -1391,10 +1391,10 @@
     <t xml:space="preserve">All WaterPaths modeling code used to simulate Triangle water supply decision-making can be found at https://github.com/bernardoct/WaterPaths/tree/JLWTPAgreementsModel. All additional modeling code, input and output data for producing the results of this manuscript can be accessed at https://www.hydroshare.org/resource/3fc8e01960d948a2bd38189dd4e7fa69/.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://github.com/bernardoct/WaterPaths/tree/JLWTPAgreementsModel", "https://www.hydroshare.org/resource/3fc8e01960d948a2bd38189dd4e7fa69")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("waterutility", "cooperation", "demand", "deepuncertainty", "optimization", "financialrisk")</t>
+    <t xml:space="preserve">https://github.com/bernardoct/WaterPaths/tree/JLWTPAgreementsModel; https://www.hydroshare.org/resource/3fc8e01960d948a2bd38189dd4e7fa69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">waterutility; cooperation; demand; deepuncertainty; optimization; financialrisk</t>
   </si>
   <si>
     <t xml:space="preserve">https://agupubs.onlinelibrary.wiley.com/doi/full/10.1029/2021EF002139</t>
@@ -1421,10 +1421,10 @@
     <t xml:space="preserve">Data and code used in the analyses are freely available on GitHub (https://github.com/acgold/HTF-on-roads) and Zenodo.org (https://doi.org/10.5281/zenodo.5562568).</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://github.com/acgold/HTF-on-roads", "https://doi.org/10.5281/zenodo.5562568")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("coastaldevelopment", "stormwatermanagement", "infrastructure", "inundationmodeling", "high-tideflooding")</t>
+    <t xml:space="preserve">https://github.com/acgold/HTF-on-roads; https://doi.org/10.5281/zenodo.5562568</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coastaldevelopment; stormwatermanagement; infrastructure; inundationmodeling; high-tideflooding</t>
   </si>
   <si>
     <t xml:space="preserve">https://onlinelibrary.wiley.com/doi/full/10.1002/esp.5495</t>
@@ -1457,7 +1457,7 @@
     <t xml:space="preserve">in paper or supp</t>
   </si>
   <si>
-    <t xml:space="preserve">c("erosion", "land-usechange", "legacysediment", "slope-areatreshold", ".", "soilnutrients", "streamchannelinitiation")</t>
+    <t xml:space="preserve">erosion; land-usechange; legacysediment; slope-areatreshold; .; soilnutrients; streamchannelinitiation</t>
   </si>
   <si>
     <t xml:space="preserve">https://onlinelibrary.wiley.com/doi/abs/10.1111/psj.12473</t>
@@ -1469,7 +1469,7 @@
     <t xml:space="preserve">External drivers of participation in regional collaborative water planning</t>
   </si>
   <si>
-    <t xml:space="preserve">c("collaborativegovernance", "policybeliefs", "regionalwaterplanning", "Gobernanzacolaborativa", "creenciaspolíticas", "planificaciónregionaldelagua", "协作治理", "政策信念", "区域水资源规划")</t>
+    <t xml:space="preserve">collaborativegovernance; policybeliefs; regionalwaterplanning; Gobernanzacolaborativa; creenciaspolíticas; planificaciónregionaldelagua; 协作治理; 政策信念; 区域水资源规划</t>
   </si>
   <si>
     <t xml:space="preserve">https://onlinelibrary.wiley.com/doi/epdf/10.1002/anie.202208150</t>
@@ -1526,7 +1526,7 @@
     <t xml:space="preserve">https://www.hydroshare.org/resource/957475e1101346a6a1cbbb62f17e747d</t>
   </si>
   <si>
-    <t xml:space="preserve">c("biology-geologyfeebacks", "DMQ99", "evapotranspiration", "headwaterstreams", "landusechange", "seasonalflashiness", "specificconductance", "streamgauges")</t>
+    <t xml:space="preserve">biology-geologyfeebacks; DMQ99; evapotranspiration; headwaterstreams; landusechange; seasonalflashiness; specificconductance; streamgauges</t>
   </si>
   <si>
     <t xml:space="preserve">https://scholar.google.com/scholar_url?url=https://ajph.aphapublications.org/doi/pdf/10.2105/AJPH.2022.307003%3Fdownload%3Dtrue&amp;hl=en&amp;sa=X&amp;d=3962241131938486649&amp;ei=H1Q7Y6aFPO2KywSS3bH4Bg&amp;scisig=AAGBfm3Q4X2sCbJJGTgTcSrsGU_FdUVJcw&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:7463423130094204642:AAGBfm306n8jEm7p9E06Y9mqflGSBiV6Pg&amp;html=&amp;pos=0&amp;folt=kw-top</t>
@@ -1577,7 +1577,7 @@
     <t xml:space="preserve">0000-0001-6231-9437</t>
   </si>
   <si>
-    <t xml:space="preserve">c("WASP", "environmentalmodeling", "nanocopper", "nanomaterials", "freswater")</t>
+    <t xml:space="preserve">WASP; environmentalmodeling; nanocopper; nanomaterials; freswater</t>
   </si>
   <si>
     <t xml:space="preserve">https://scholar.google.com/scholar_url?url=https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/hir.12445&amp;hl=en&amp;sa=X&amp;d=7293212103073901469&amp;ei=2fm2YrzQKtHjmQGNwb84&amp;scisig=AAGBfm1zjx3-V2aCgS0L1xZx26MYDvF-tg&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:3552202248086981277:AAGBfm3xoOKMdpREzJ__fgBb7pdlMpLHFA&amp;html=&amp;pos=1&amp;folt=kw</t>
@@ -1598,7 +1598,7 @@
     <t xml:space="preserve">0000-0001-7360-0021</t>
   </si>
   <si>
-    <t xml:space="preserve">c("healtheducation", "healthinformationneeds", "healthprofessionals", "informationdissemination", "informationliteracy", "informationseekingbehavior", "patienteducation", "research", "qualitative")</t>
+    <t xml:space="preserve">healtheducation; healthinformationneeds; healthprofessionals; informationdissemination; informationliteracy; informationseekingbehavior; patienteducation; research; qualitative</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/ivRR62</t>
@@ -1649,7 +1649,7 @@
     <t xml:space="preserve">0000-0002-6373-8374</t>
   </si>
   <si>
-    <t xml:space="preserve">c("crAssphage", "Municipaluntreatedwastewater", "Temporalvariations", "Spatialvariations", "Entericpathogenscorrelations", "Bacteria", "Andviruses", ";", "qPCR", "rt-qPCR")</t>
+    <t xml:space="preserve">crAssphage; Municipaluntreatedwastewater; Temporalvariations; Spatialvariations; Entericpathogenscorrelations; Bacteria; Andviruses; ;; qPCR; rt-qPCR</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/36633899/</t>
@@ -1703,7 +1703,7 @@
     <t xml:space="preserve">The codes used in this research are available from the authors upon request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("ArtificialNeuralNetworks", "Geneticprogramming", "Antedcedentenvironmentalconditions", "Temperature", "Salinity", "Oysters")</t>
+    <t xml:space="preserve">ArtificialNeuralNetworks; Geneticprogramming; Antedcedentenvironmentalconditions; Temperature; Salinity; Oysters</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubmed.ncbi.nlm.nih.gov/36356280/</t>
@@ -1742,11 +1742,10 @@
     <t xml:space="preserve">The raw sequencing data (FASTQ) generated in this study have been deposited in the European Nucleotide Archive and can be accessed without restrictions. The data from major sampling rounds have the following project accession numbers: PRJEB40798, PRJEB40816, PRJEB40815 and PRJEB27621. Sequencing data from the longitudinal city sampling sites are deposited under PRJEB51229, while the included datasets from the previous study are deposited under ERP015409. See Supplementary Data 1 for exact sample, experiment and run accessions. Source data are provided with this paper. This study also utilized the publicly available databases of ResFinder, PLSDB, Silva and Kraken 2.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://www.ebi.ac.uk/ena/browser/view/PRJEB40798", "https://www.ebi.ac.uk/ena/browser/view/PRJEB40816", "https://www.ebi.ac.uk/ena/browser/view/PRJEB40815", "https://www.ebi.ac.uk/ena/browser/view/PRJEB27621", "https://www.ebi.ac.uk/ena/browser/view/PRJEB51229", "https://www.ebi.ac.uk/ena/browser/view/ERP015409", "https://bitbucket.org/genomicepidemiology/resfinder_db", "https://ccb-microbe.cs.uni-saarland.de/plsdb/plasmids/download/", "https://www.arb-silva.de/download/arb-files/", "https://benlangmead.github.io/aws-indexes/k2"
-)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Antimicrobialresistance", "Metagenomics", "Microbialecology", "Policyandpublichealthinmicrobiology")</t>
+    <t xml:space="preserve">https://www.ebi.ac.uk/ena/browser/view/PRJEB40798; https://www.ebi.ac.uk/ena/browser/view/PRJEB40816; https://www.ebi.ac.uk/ena/browser/view/PRJEB40815; https://www.ebi.ac.uk/ena/browser/view/PRJEB27621; https://www.ebi.ac.uk/ena/browser/view/PRJEB51229; https://www.ebi.ac.uk/ena/browser/view/ERP015409; https://bitbucket.org/genomicepidemiology/resfinder_db; https://ccb-microbe.cs.uni-saarland.de/plsdb/plasmids/download/; https://www.arb-silva.de/download/arb-files/; https://benlangmead.github.io/aws-indexes/k2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antimicrobialresistance; Metagenomics; Microbialecology; Policyandpublichealthinmicrobiology</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.nature.com/articles/s41370-022-00475-0</t>
@@ -1773,7 +1772,7 @@
     <t xml:space="preserve">The datasets generated during and/or analyzed during the current study are available from the corresponding author on reasonable request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Pretermbirth", "Lowbirthweight", "Adversebirthoutcome", "Pollutedsites", "Superfund", "Industrialsites")</t>
+    <t xml:space="preserve">Pretermbirth; Lowbirthweight; Adversebirthoutcome; Pollutedsites; Superfund; Industrialsites</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.nature.com/articles/s43247-022-00501-x</t>
@@ -1812,7 +1811,7 @@
     <t xml:space="preserve">https://doi.org/10.6084/m9.figshare.20137649.v265</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Carboncycle", "Climate-changemitigation", "Environmentalimpact")</t>
+    <t xml:space="preserve">Carboncycle; Climate-changemitigation; Environmentalimpact</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.nature.com/articles/s41545-021-00128-z</t>
@@ -1845,7 +1844,7 @@
     <t xml:space="preserve">no data generated</t>
   </si>
   <si>
-    <t xml:space="preserve">c("ChemicalEngineering", "Waterresources")</t>
+    <t xml:space="preserve">ChemicalEngineering; Waterresources</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.nature.com/articles/s41597-022-01358-7</t>
@@ -1876,10 +1875,10 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://github.com/TransformingDrainageProject/Drain-Flow-Gap-Filling", "https://github.com/isudatateam/datateam")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Agriculture", "Environmentalimpact", "Hydrology", "Waterresources")</t>
+    <t xml:space="preserve">https://github.com/TransformingDrainageProject/Drain-Flow-Gap-Filling; https://github.com/isudatateam/datateam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agriculture; Environmentalimpact; Hydrology; Waterresources</t>
   </si>
   <si>
     <t xml:space="preserve">https://journals.plos.org/plosntds/article?id=10.1371/journal.pntd.0011496</t>
@@ -1948,7 +1947,7 @@
     <t xml:space="preserve">Field performance of the GaugeCam image-based water level measurement system</t>
   </si>
   <si>
-    <t xml:space="preserve">c("docx", "tif")</t>
+    <t xml:space="preserve">docx; tif</t>
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.1371/journal.pwat.0000032.s001</t>
@@ -2077,7 +2076,7 @@
     <t xml:space="preserve">mark_sobsey@unc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Cryptosporidium", "Bacillusspores", "MS2coliphage", "bromine", "chlorine", "disinfection", "watertreatment")</t>
+    <t xml:space="preserve">Cryptosporidium; Bacillusspores; MS2coliphage; bromine; chlorine; disinfection; watertreatment</t>
   </si>
   <si>
     <t xml:space="preserve">32</t>
@@ -2110,7 +2109,7 @@
     <t xml:space="preserve">0000-0003-1315-1791</t>
   </si>
   <si>
-    <t xml:space="preserve">c("PFASdestruction", "fluoroethers", "GenX", "Nafionbyproduct2", "photolysis")</t>
+    <t xml:space="preserve">PFASdestruction; fluoroethers; GenX; Nafionbyproduct2; photolysis</t>
   </si>
   <si>
     <t xml:space="preserve">35</t>
@@ -2149,10 +2148,10 @@
     <t xml:space="preserve">The storm drain water level data used for flood detection and analysis in the study are archived on Zenodo (https://doi.org/10.5281/zenodo.7135955) and can also be downloaded from our project web app (https://sunnydayflood.apps.cloudapps.unc.edu). The software for the SuDS sensor framework are available on GitHub (https://github.com/sunny-day-flooding-project) and tutorials are archived on Zenodo (Hayden-Lowe et al., 2022, https://doi.org/10.5281/zenodo.7017187).</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://doi.org/10.5281/zenodo.7135955", "https://sunnydayflood.apps.cloudapps.unc.edu", "https://github.com/sunny-day-flooding-project", "https://doi.org/10.5281/zenodo.7017187")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("coastalflooding", "low-costsensors", "hightideflooding", "stormwatermanagement", "coastalinfrastructure", "sealevelrise")</t>
+    <t xml:space="preserve">https://doi.org/10.5281/zenodo.7135955; https://sunnydayflood.apps.cloudapps.unc.edu; https://github.com/sunny-day-flooding-project; https://doi.org/10.5281/zenodo.7017187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coastalflooding; low-costsensors; hightideflooding; stormwatermanagement; coastalinfrastructure; sealevelrise</t>
   </si>
   <si>
     <t xml:space="preserve">39</t>
@@ -2164,7 +2163,7 @@
     <t xml:space="preserve">Affordability of household water services across the United States</t>
   </si>
   <si>
-    <t xml:space="preserve">c("docx", "csv")</t>
+    <t xml:space="preserve">docx; csv</t>
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.1371/journal.pwat.0000123.s001</t>
@@ -2209,7 +2208,7 @@
     <t xml:space="preserve">Anonymized data can be shared upon request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("PFAS", "Drinkingwater", "USEPA", "PFPrA", "Ultra-shortchain")</t>
+    <t xml:space="preserve">PFAS; Drinkingwater; USEPA; PFPrA; Ultra-shortchain</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2306-5338/10/7/156</t>
@@ -2242,7 +2241,7 @@
     <t xml:space="preserve">Raw data can be provided upon request by emailing the corresponding author at Humphreyc@ecu.edu.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("coastal", "fecalbacteria", "runoff", "stormwater")</t>
+    <t xml:space="preserve">coastal; fecalbacteria; runoff; stormwater</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2073-4441/15/13/2436</t>
@@ -2269,7 +2268,7 @@
     <t xml:space="preserve">The data presented in this study are available on request from the corresponding author.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("cyanobacteria", "cyanotoxin", "microcystin", "stormwaterpollution", "eutrophication")</t>
+    <t xml:space="preserve">cyanobacteria; cyanotoxin; microcystin; stormwaterpollution; eutrophication</t>
   </si>
   <si>
     <t xml:space="preserve">http://eepurl.com/ikRgmb</t>
@@ -2296,7 +2295,7 @@
     <t xml:space="preserve">0000-0002-0944-8632</t>
   </si>
   <si>
-    <t xml:space="preserve">c("waterscarcity", "waterrecycling", "wastewatertreatmentplants", "nutrients", "phosphorus")</t>
+    <t xml:space="preserve">waterscarcity; waterrecycling; wastewatertreatmentplants; nutrients; phosphorus</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/1422-0067/24/2/1295</t>
@@ -2335,7 +2334,7 @@
     <t xml:space="preserve">Data included in this study are available from the corresponding author upon reasonable request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("HWTS", "POU", "chitosan", "coagulation", "sandfiltration", "bacterialreduction", "virusreduction")</t>
+    <t xml:space="preserve">HWTS; POU; chitosan; coagulation; sandfiltration; bacterialreduction; virusreduction</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2073-4441/14/13/2088</t>
@@ -2362,7 +2361,7 @@
     <t xml:space="preserve">jozo@sfsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("explainability", "LSPmethod", "waterquality", "decision-making")</t>
+    <t xml:space="preserve">explainability; LSPmethod; waterquality; decision-making</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2306-5338/9/12/218</t>
@@ -2389,10 +2388,10 @@
     <t xml:space="preserve">All publicly available datasets used in this research are available at the locations indicated in Table 1 or upon request in their processed version from the corresponding author.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://coast.noaa.gov/slrdata/", "https://coast.noaa.gov/slrdata/", "https://fris.nc.gov/fris/Home.aspx?ST=NC", "https://earthexplorer.usgs.gov/", "https://deq.nc.gov/about/divisions/coastal", "https://www.nconemap.gov/pages/parcels")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("wetlands", "nature-basedsolutions", "floodmitigation", "coastalflooding", "tidalwatersheds")</t>
+    <t xml:space="preserve">https://coast.noaa.gov/slrdata/; https://coast.noaa.gov/slrdata/; https://fris.nc.gov/fris/Home.aspx?ST=NC; https://earthexplorer.usgs.gov/; https://deq.nc.gov/about/divisions/coastal; https://www.nconemap.gov/pages/parcels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wetlands; nature-basedsolutions; floodmitigation; coastalflooding; tidalwatersheds</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2076-3417/12/19/10159/pdf?version=1665394404</t>
@@ -2407,7 +2406,7 @@
     <t xml:space="preserve">https://www.mdpi.com/article/10.3390/app121910159/s1</t>
   </si>
   <si>
-    <t xml:space="preserve">c("reclaimedwater", "waterreuse", "water-supplysystems", "agro-wastewater", "riskassessment")</t>
+    <t xml:space="preserve">reclaimedwater; waterreuse; water-supplysystems; agro-wastewater; riskassessment</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2073-445X/11/9/1504/htm</t>
@@ -2437,10 +2436,10 @@
     <t xml:space="preserve">The data presented in this study are available in Appendix A.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://www.nconemap.gov/", "https://www.nrcs.usda.gov/wps/portal/nrcs/detail/soils/survey/geo/?cid=nrcs142p2_053628", "https://www.nconemap.gov/", "https://www.nconemap.gov/")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("geospatialanalysis", "landsuitability", "floodmitigation", "nature-basedsolutions(NBS)", "rurallandscapes", "GeographicInformationSystems(GIS)", "floodresilience")</t>
+    <t xml:space="preserve">https://www.nconemap.gov/; https://www.nrcs.usda.gov/wps/portal/nrcs/detail/soils/survey/geo/?cid=nrcs142p2_053628; https://www.nconemap.gov/; https://www.nconemap.gov/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geospatialanalysis; landsuitability; floodmitigation; nature-basedsolutions(NBS); rurallandscapes; GeographicInformationSystems(GIS); floodresilience</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2076-3417/12/19/10159</t>
@@ -2461,7 +2460,7 @@
     <t xml:space="preserve">Data are summarized and displayed in figures. Raw data may be made available via email with the corresponding author.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("coastal", "eutrophicationsepticsystems")</t>
+    <t xml:space="preserve">coastal; eutrophicationsepticsystems</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2073-4441/14/10/1525/pdf?version=1652171768</t>
@@ -2479,7 +2478,7 @@
     <t xml:space="preserve">jdyer@geosci.msstate.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("hydrologicdrought", "SoutheastUS", "NationalWaterModel")</t>
+    <t xml:space="preserve">hydrologicdrought; SoutheastUS; NationalWaterModel</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/1660-4601/19/8/4628/pdf</t>
@@ -2509,10 +2508,10 @@
     <t xml:space="preserve">The data for socioeconomic vulnerability variables can be found through API of American Community Survey [62]. Data for community access to safe drinking water are openly available at Safe Drinking Water Information System (SDWIS) [63]. Land cover raster maps of 2019 and 2016 can be found at Multi-Resolution Land Characteristic Consortium (MRLC) website [64]. To access drought data, we used the Comprehensive Statistics page of Data Download section of U.S. Drought Monitor [65]. The data that support the findings of this study are openly available in Mendeley Data [66].</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://www.census.gov/data/developers/data-sets/acs-5year.html", "https://www.epa.gov/ground-water-and-drinking-water/safe-drinking-water-information-system-sdwis-federal-reporting")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("droughtandhealth", "droughtrisk", "LocalMoran", "sI", "droughtvulnerability", "U.S.drought")</t>
+    <t xml:space="preserve">https://www.census.gov/data/developers/data-sets/acs-5year.html; https://www.epa.gov/ground-water-and-drinking-water/safe-drinking-water-information-system-sdwis-federal-reporting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">droughtandhealth; droughtrisk; LocalMoran; sI; droughtvulnerability; U.S.drought</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2071-1050/14/7/3889/pdf</t>
@@ -2539,7 +2538,7 @@
     <t xml:space="preserve">0000-0002-2834-3764</t>
   </si>
   <si>
-    <t xml:space="preserve">c("environmentalplanning", "policyevaluation", "riparianbuffers")</t>
+    <t xml:space="preserve">environmentalplanning; policyevaluation; riparianbuffers</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/1999-4907/13/3/411</t>
@@ -2572,7 +2571,7 @@
     <t xml:space="preserve">https://github.com/hkqcqq/CoastalWetlandDetection.git</t>
   </si>
   <si>
-    <t xml:space="preserve">c("coastalwetlanddegradation", "remotesensing", "NDVI", "climatechange", "sea-levelrise", "saltwaterintrusion", "hydrologicmodel", "AlligatorRiverNationalWildlifeRefuge", "USA")</t>
+    <t xml:space="preserve">coastalwetlanddegradation; remotesensing; NDVI; climatechange; sea-levelrise; saltwaterintrusion; hydrologicmodel; AlligatorRiverNationalWildlifeRefuge; USA</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdpi.com/2073-4441/14/2/247</t>
@@ -2602,7 +2601,7 @@
     <t xml:space="preserve">https://doi.org/10.7910/DVN/0ETQ74</t>
   </si>
   <si>
-    <t xml:space="preserve">c("waterinfrastructure", "waterservices", "waterutilities", "waterbills", "billingfrequency", "customerassistanceprograms(CAPS)", "affordability")</t>
+    <t xml:space="preserve">waterinfrastructure; waterservices; waterutilities; waterbills; billingfrequency; customerassistanceprograms(CAPS); affordability</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.3c01146</t>
@@ -2629,7 +2628,7 @@
     <t xml:space="preserve">0000-0003-2954-1110</t>
   </si>
   <si>
-    <t xml:space="preserve">c("canine", "drinkingwater", "equine", "fluoroether", "OneHealth", "nafionby-product2", "GenXchemicals", "PFOA", "PFOS")</t>
+    <t xml:space="preserve">canine; drinkingwater; equine; fluoroether; OneHealth; nafionby-product2; GenXchemicals; PFOA; PFOS</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.estlett.0c00255</t>
@@ -2653,7 +2652,7 @@
     <t xml:space="preserve">0000-0002-5289-1218</t>
   </si>
   <si>
-    <t xml:space="preserve">c("drinkingwater", "fluoropolymers", "food", "safety", "toxins")</t>
+    <t xml:space="preserve">drinkingwater; fluoropolymers; food; safety; toxins</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.estlett.3c00487</t>
@@ -2665,7 +2664,7 @@
     <t xml:space="preserve">jmacdon@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Airpollution", "Color", "Environmentalpollution", "Environmentalscience", "Impurities")</t>
+    <t xml:space="preserve">Airpollution; Color; Environmentalpollution; Environmentalscience; Impurities</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.2c07477</t>
@@ -2674,7 +2673,7 @@
     <t xml:space="preserve">Improved Decision Making for Water Lead Testing in U.S. Child Care Facilities Using Machine-Learned Bayesian Networks</t>
   </si>
   <si>
-    <t xml:space="preserve">c("pdf", "html")</t>
+    <t xml:space="preserve">pdf; html</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.2c07477?goto=supporting-info</t>
@@ -2698,7 +2697,7 @@
     <t xml:space="preserve">https://doi.org/10.5281/zenodo.7477787</t>
   </si>
   <si>
-    <t xml:space="preserve">c("lead", "Children", "shealth", "drinkingwater", "machinelearning", "riskassessment")</t>
+    <t xml:space="preserve">lead; Children; shealth; drinkingwater; machinelearning; riskassessment</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/full/10.1021/acs.est.2c07316</t>
@@ -2728,7 +2727,7 @@
     <t xml:space="preserve">0000-0001-6220-8673</t>
   </si>
   <si>
-    <t xml:space="preserve">c("PFASair-waterinterfacialadsorption", "QSPR", "nonequilibrium", "unsaturatedcolumns", "panfilm")</t>
+    <t xml:space="preserve">PFASair-waterinterfacialadsorption; QSPR; nonequilibrium; unsaturatedcolumns; panfilm</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.accounts.2c00591</t>
@@ -2749,7 +2748,7 @@
     <t xml:space="preserve">soobare@ncat.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("adsorption", "molecules", "nanofibers", "remediation")</t>
+    <t xml:space="preserve">adsorption; molecules; nanofibers; remediation</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acsestwater.2c00320</t>
@@ -2779,7 +2778,7 @@
     <t xml:space="preserve">0000-0001-5246-2213</t>
   </si>
   <si>
-    <t xml:space="preserve">c("nontargetedanalysis", "anthropogenicchemicals", "wastewater", "landfillleachate", "reverseosmosis")</t>
+    <t xml:space="preserve">nontargetedanalysis; anthropogenicchemicals; wastewater; landfillleachate; reverseosmosis</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/full/10.1021/acs.estlett.2c00502?cookieSet=1</t>
@@ -2812,7 +2811,7 @@
     <t xml:space="preserve">0000-0001-5223-2848</t>
   </si>
   <si>
-    <t xml:space="preserve">c("per-andpolyfluoroalkylsubstances(PFAS)", "presumptivecontamination", "PFAStestingandinvestigation", "AFFF", "PFASwasteanddisposal")</t>
+    <t xml:space="preserve">per-andpolyfluoroalkylsubstances(PFAS); presumptivecontamination; PFAStestingandinvestigation; AFFF; PFASwasteanddisposal</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/full/10.1021/acsestwater.2c00287?cookieSet=1</t>
@@ -2833,7 +2832,7 @@
     <t xml:space="preserve">0000-0001-9488-8124</t>
   </si>
   <si>
-    <t xml:space="preserve">c("anatomy", "genetics", "infectiousdiseases", "viruses", "wastewater")</t>
+    <t xml:space="preserve">anatomy; genetics; infectiousdiseases; viruses; wastewater</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.2c04717?cookieSet=1</t>
@@ -2863,7 +2862,7 @@
     <t xml:space="preserve">0000-0001-8928-0157</t>
   </si>
   <si>
-    <t xml:space="preserve">c("coalash", "lacustrinesediment", "multiproxytracing", "aquaticecosystems")</t>
+    <t xml:space="preserve">coalash; lacustrinesediment; multiproxytracing; aquaticecosystems</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.2c03076</t>
@@ -2884,7 +2883,7 @@
     <t xml:space="preserve">0000-0003-1966-2680</t>
   </si>
   <si>
-    <t xml:space="preserve">c("waterandsanitationinfrastructure", "disadvantagedunincorporatedcommunities", "environmetaljustice", "participatoryprocess", "sociotechnicaldesign")</t>
+    <t xml:space="preserve">waterandsanitationinfrastructure; disadvantagedunincorporatedcommunities; environmetaljustice; participatoryprocess; sociotechnicaldesign</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/abs/10.1021/acsapm.2c00959</t>
@@ -2914,7 +2913,7 @@
     <t xml:space="preserve">0000-0003-3395-4823</t>
   </si>
   <si>
-    <t xml:space="preserve">c("textiledyes", "environmentalpollution", "cleanwater", "sustainability", "polycarbodiimide", "topologicalpolarsurfacearea(TPSA)", "moleculartransport")</t>
+    <t xml:space="preserve">textiledyes; environmentalpollution; cleanwater; sustainability; polycarbodiimide; topologicalpolarsurfacearea(TPSA); moleculartransport</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.2c00224</t>
@@ -2941,7 +2940,7 @@
     <t xml:space="preserve">marc_serre@unc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("land-useregression", "molecularmicrobialsourcetracking", "surfacewater", "sediment", "rivernetworks", "animalfeedingoperations", "septicsystems")</t>
+    <t xml:space="preserve">land-useregression; molecularmicrobialsourcetracking; surfacewater; sediment; rivernetworks; animalfeedingoperations; septicsystems</t>
   </si>
   <si>
     <t xml:space="preserve">https://pubs.acs.org/doi/10.1021/acs.est.1c05683</t>
@@ -2962,7 +2961,7 @@
     <t xml:space="preserve">swdaly@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("multiplewatersourceuse", "supplementalunimprovedsourceuse", "fecalcontamination", "MonteCarlosimulations", "drinkingwaterquality", "low-andmiddle-incomecountries")</t>
+    <t xml:space="preserve">multiplewatersourceuse; supplementalunimprovedsourceuse; fecalcontamination; MonteCarlosimulations; drinkingwaterquality; low-andmiddle-incomecountries</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0043135423005481</t>
@@ -2992,7 +2991,7 @@
     <t xml:space="preserve">Data will be made available on request</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Microplasticsinrivers", "Watermanagement", "DiversionsAbstraction", "Pairedcatchmentapproach", "Globalmodels")</t>
+    <t xml:space="preserve">Microplasticsinrivers; Watermanagement; DiversionsAbstraction; Pairedcatchmentapproach; Globalmodels</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0925857423001209</t>
@@ -3016,7 +3015,7 @@
     <t xml:space="preserve">curtr@duke.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Pocosin", "Carbon", "Methane", "GHG", "Netecosystemexchange", "Hydrologicrestoration", "Peatland", "Evergreenshrubbog", "Watertabledepth", "Eddycovariance", "", "Carbondioxide")</t>
+    <t xml:space="preserve">Pocosin; Carbon; Methane; GHG; Netecosystemexchange; Hydrologicrestoration; Peatland; Evergreenshrubbog; Watertabledepth; Eddycovariance; Carbondioxide</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969723037142</t>
@@ -3040,7 +3039,7 @@
     <t xml:space="preserve">sam.hall@alumni.duke.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Per-andpolyfluoroalkylsubstances", "PFAS", "Drinkingwater", "Serum", "Humanhealthoutcomes")</t>
+    <t xml:space="preserve">Per-andpolyfluoroalkylsubstances; PFAS; Drinkingwater; Serum; Humanhealthoutcomes</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0160412023003069?via%3Dihub</t>
@@ -3070,10 +3069,10 @@
     <t xml:space="preserve">All data are available. All data presented can be found in a series of USGS data releases (Meppelink et al., 2022, Romanok and Bradley, 2018, Romanok and Bradley, 2021, Romanok et al., 2022, Romanok et al., 2019, Romanok et al., 2023a, Romanok et al., 2023b, Romanok et al., 2023c). For links to the individual USGS data releases see Table S1.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://www.sciencebase.gov/catalog/item/5fad56aad34eb413d5df459c", "https://www.sciencebase.gov/catalog/item/5ab3d60be4b081f61ab5e3d4")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Per-andpolyfluoroalkylsubstances", "Drinking-water", "Public-supply", "Private-wellsSources", "Healtheffect")</t>
+    <t xml:space="preserve">https://www.sciencebase.gov/catalog/item/5fad56aad34eb413d5df459c; https://www.sciencebase.gov/catalog/item/5ab3d60be4b081f61ab5e3d4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-andpolyfluoroalkylsubstances; Drinking-water; Public-supply; Private-wellsSources; Healtheffect</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0043135423005523?via%3Dihub</t>
@@ -3103,7 +3102,7 @@
     <t xml:space="preserve">cstauber@gsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Zikavirus", "wastewater-basedepidemiology", "resource-constrainedsettings")</t>
+    <t xml:space="preserve">Zikavirus; wastewater-basedepidemiology; resource-constrainedsettings</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S2213343723012411?via%3Dihub</t>
@@ -3136,7 +3135,7 @@
     <t xml:space="preserve">No data was used for the research described in the article.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Airpollutioncontrol", "Biologicalgastreatment", "Capillaryreactor", "Hydrophobicpollutants", "Segmentedflow")</t>
+    <t xml:space="preserve">Airpollutioncontrol; Biologicalgastreatment; Capillaryreactor; Hydrophobicpollutants; Segmentedflow</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969723027080?via%3Dihub</t>
@@ -3157,7 +3156,7 @@
     <t xml:space="preserve">ylai5@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Marinemicroalgae", "Dunaliellaviridis", "Flocculation", "Harvesting", "Waterreuse", "Dissolvedorganicmatter")</t>
+    <t xml:space="preserve">Marinemicroalgae; Dunaliellaviridis; Flocculation; Harvesting; Waterreuse; Dissolvedorganicmatter</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0277379123002019</t>
@@ -3184,10 +3183,10 @@
     <t xml:space="preserve">Data are reposited at www.neotomadb.org and https://www.ncei.noaa.gov. Code for analogs and paleoclimate reconstructions are available at https://github.com/davidfastovich/gds_climate_reconstruction.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("https://www.ncei.noaa.gov", "https://github.com/davidfastovich/gds_climate_reconstruction")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c("Palynology", "Plantmacrofossil", "Charcoal", "Paleoclimatereconstruction", "Sea-levelrise", "Wildfire", "Wetlanddevelopment", "Hydroperiod")</t>
+    <t xml:space="preserve">https://www.ncei.noaa.gov; https://github.com/davidfastovich/gds_climate_reconstruction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palynology; Plantmacrofossil; Charcoal; Paleoclimatereconstruction; Sea-levelrise; Wildfire; Wetlanddevelopment; Hydroperiod</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969723018855</t>
@@ -3208,7 +3207,7 @@
     <t xml:space="preserve">The data will be posted at https://catalog.data.gov/dataset and available upon request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Microbiome", "Outdoorair", "Greenspace", "AirborneBacteria", "16SrRNA", "Aerobiome")</t>
+    <t xml:space="preserve">Microbiome; Outdoorair; Greenspace; AirborneBacteria; 16SrRNA; Aerobiome</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S2214109X23000062?via%3Dihub</t>
@@ -3250,7 +3249,7 @@
     <t xml:space="preserve">a.sohns@northeastern.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Watersecurity", "Textanalysis", "Structuraltopicmodeling", "Planning", "Environmentaljustice")</t>
+    <t xml:space="preserve">Watersecurity; Textanalysis; Structuraltopicmodeling; Planning; Environmentaljustice</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S004313542300444X?via%3Dihub</t>
@@ -3262,7 +3261,7 @@
     <t xml:space="preserve">0000-0001-8935-7759</t>
   </si>
   <si>
-    <t xml:space="preserve">c("crAssphage", "Municipaluntreatedwastewater", "Temporalvariations", "Spatialvariations", "Entericpathogenscorrelations", "Bacteria", "Andviruses", "qPCR", "rt-qPCR")</t>
+    <t xml:space="preserve">crAssphage; Municipaluntreatedwastewater; Temporalvariations; Spatialvariations; Entericpathogenscorrelations; Bacteria; Andviruses; qPCR; rt-qPCR</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969723000414</t>
@@ -3289,7 +3288,7 @@
     <t xml:space="preserve">not shareable</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Groundwatercontamination", "Swinelagoons", "Privatewells", "Atmosphericstressors", "Environmentalpollution")</t>
+    <t xml:space="preserve">Groundwatercontamination; Swinelagoons; Privatewells; Atmosphericstressors; Environmentalpollution</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969723015565?via%3Dihub</t>
@@ -3310,7 +3309,7 @@
     <t xml:space="preserve">jjkurkif@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Microplastics", "Streamflow", "Urbandevelopment", "Sediment", "Watershed", "Samplingmethod")</t>
+    <t xml:space="preserve">Microplastics; Streamflow; Urbandevelopment; Sediment; Watershed; Samplingmethod</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S1470160X23003321</t>
@@ -3337,7 +3336,7 @@
     <t xml:space="preserve">0000-0002-2843-4965</t>
   </si>
   <si>
-    <t xml:space="preserve">c("UAV", "UAS", "Rugosity", "Geomorphometry", "Coastalhabitat", "Remotesensing")</t>
+    <t xml:space="preserve">UAV; UAS; Rugosity; Geomorphometry; Coastalhabitat; Remotesensing</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S2589537023001359</t>
@@ -3349,7 +3348,7 @@
     <t xml:space="preserve">Environmental cleaning to prevent hospital-acquired infections on non-intensive care units: a pragmatic, single-centre, cluster randomized controlled, crossover trial comparing soap-based, disinfection and probiotic cleaning</t>
   </si>
   <si>
-    <t xml:space="preserve">c("docx", "pdf")</t>
+    <t xml:space="preserve">docx; pdf</t>
   </si>
   <si>
     <t xml:space="preserve">https://ars.els-cdn.com/content/image/1-s2.0-S2589537023001359-mmc1.docx</t>
@@ -3367,7 +3366,7 @@
     <t xml:space="preserve">0000-0002-1225-9023</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Hospital-aquiredinfection", "Multidrug-resistantpathogen", "Environmentalcleaning", "Probiotic", "Randomized-controlledtrial", "Environmentalhygiene", "MRSAVRE", "Multidrug-resistantGram-negative")</t>
+    <t xml:space="preserve">Hospital-aquiredinfection; Multidrug-resistantpathogen; Environmentalcleaning; Probiotic; Randomized-controlledtrial; Environmentalhygiene; MRSAVRE; Multidrug-resistantGram-negative</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0377026523000155</t>
@@ -3391,7 +3390,7 @@
     <t xml:space="preserve">0000-0001-6309-1403</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Atmosphericforcing", "CapeHatteras", "PEACH", "Atmosphericcyclones", "Atmosphericwarmandcoolseasons")</t>
+    <t xml:space="preserve">Atmosphericforcing; CapeHatteras; PEACH; Atmosphericcyclones; Atmosphericwarmandcoolseasons</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969723017424</t>
@@ -3418,7 +3417,7 @@
     <t xml:space="preserve">mriza@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Contamination", "Distribution", "Environment", "Healthimpact", "NorthCarolina", "PFASsources")</t>
+    <t xml:space="preserve">Contamination; Distribution; Environment; Healthimpact; NorthCarolina; PFASsources</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0169555X23000867</t>
@@ -3439,7 +3438,7 @@
     <t xml:space="preserve">jdp@uky.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Landscapechange", "Climatechange", "Attribution", "NeuseRiver", "Sea-levelrise", "Marshloss")</t>
+    <t xml:space="preserve">Landscapechange; Climatechange; Attribution; NeuseRiver; Sea-levelrise; Marshloss</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722075118</t>
@@ -3460,7 +3459,7 @@
     <t xml:space="preserve">https://github.com/UNCSRP/CASS-IT</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Clustering", "Metals", "Privatewells", "Socialvulnerability", "Geographicdata")</t>
+    <t xml:space="preserve">Clustering; Metals; Privatewells; Socialvulnerability; Geographicdata</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969723000414?via%3Dihub</t>
@@ -3490,7 +3489,7 @@
     <t xml:space="preserve">0000-0003-0639-7865</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Microbioreactor", "Volatileorganiccompound", "Biofiltration", "Modeling")</t>
+    <t xml:space="preserve">Microbioreactor; Volatileorganiccompound; Biofiltration; Modeling</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0043135423000878?via%3Dihub</t>
@@ -3508,7 +3507,7 @@
     <t xml:space="preserve">Department of Civil, Construction, and Environmental Engineering, North Carolina State University, Raleigh, NC 27695, United States</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Biofiltration", "Cometabolism", "Adsorption", "Emergingcontaminants")</t>
+    <t xml:space="preserve">Biofiltration; Cometabolism; Adsorption; Emergingcontaminants</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0378377423000446</t>
@@ -3517,7 +3516,7 @@
     <t xml:space="preserve">Department of Biological and Agricultural Engineering, North Carolina State University, Raleigh, NC 27695–7625, USA</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Subsurfacedrainage", "Subirrigation", "On-farmwaterstorage", "Drainagewaterreuse", "Supplementalirrigation", "Surfacewaterquality")</t>
+    <t xml:space="preserve">Subsurfacedrainage; Subirrigation; On-farmwaterstorage; Drainagewaterreuse; Supplementalirrigation; Surfacewaterquality</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S209592732200593X?via%3Dihub</t>
@@ -3559,7 +3558,7 @@
     <t xml:space="preserve">kostas@ce.gatech.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Wastewater-basedepidemiology", "Passivesampling", "Mooreswab")</t>
+    <t xml:space="preserve">Wastewater-basedepidemiology; Passivesampling; Mooreswab</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0304389422024864</t>
@@ -3592,7 +3591,7 @@
     <t xml:space="preserve">The data that has been used is confidential.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("SARS-CoV-2", "Wastewater-basedepidemiology", "Universitycampus", "Emergingcontaminants", "Disinfectants")</t>
+    <t xml:space="preserve">SARS-CoV-2; Wastewater-basedepidemiology; Universitycampus; Emergingcontaminants; Disinfectants</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0743016722002844</t>
@@ -3616,7 +3615,7 @@
     <t xml:space="preserve">0000-0001-9333-9641</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Geographicinformationsystems", "Ruralgeography", "statisticalanalysis")</t>
+    <t xml:space="preserve">Geographicinformationsystems; Ruralgeography; statisticalanalysis</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722079372</t>
@@ -3634,7 +3633,7 @@
     <t xml:space="preserve">etgay@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Forestedwatersheds", "FUTURESmodel", "Landuselandcoverchange(LULCC)", "Hydrologicmodeling", "SoilandWaterAssessmentTool(SWAT)", "Globalclimatemodel")</t>
+    <t xml:space="preserve">Forestedwatersheds; FUTURESmodel; Landuselandcoverchange(LULCC); Hydrologicmodeling; SoilandWaterAssessmentTool(SWAT); Globalclimatemodel</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0169772222001723</t>
@@ -3664,7 +3663,7 @@
     <t xml:space="preserve">The data used are given in online supplementary material associated with the paper.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("VOC", "Contaminantflux", "Groundwater", "Stream")</t>
+    <t xml:space="preserve">VOC; Contaminantflux; Groundwater; Stream</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0378383922001880</t>
@@ -3688,7 +3687,7 @@
     <t xml:space="preserve">0000-0001-7724-5805</t>
   </si>
   <si>
-    <t xml:space="preserve">c("CoastalaltimetrySealevel", "Waves", "Videocamera", "Tidegauge", "Buoy", "Altimeter", "Significantwaveheight", "Re-trackingalgorithm")</t>
+    <t xml:space="preserve">CoastalaltimetrySealevel; Waves; Videocamera; Tidegauge; Buoy; Altimeter; Significantwaveheight; Re-trackingalgorithm</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722070966</t>
@@ -3712,7 +3711,7 @@
     <t xml:space="preserve">jill.stewart@unc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Wastewater-basedepidemiology", "Sewagesurveillance", "Coronavirus", "COVID", "ddPCR")</t>
+    <t xml:space="preserve">Wastewater-basedepidemiology; Sewagesurveillance; Coronavirus; COVID; ddPCR</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722075118?via%3Dihub</t>
@@ -3748,7 +3747,7 @@
     <t xml:space="preserve">0000-0003-4519-8156</t>
   </si>
   <si>
-    <t xml:space="preserve">c("GHGEmissions", "Waterextractable", "Phosphorus", "Zinc", "Copper", "NorthCarolina")</t>
+    <t xml:space="preserve">GHGEmissions; Waterextractable; Phosphorus; Zinc; Copper; NorthCarolina</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S2590061722000539</t>
@@ -3769,7 +3768,7 @@
     <t xml:space="preserve">wcurtis1@citadel.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Risk", "Compoundhazard", "Flood", "Rural", "Emergencymanagement", "Planning", "CCWE")</t>
+    <t xml:space="preserve">Risk; Compoundhazard; Flood; Rural; Emergencymanagement; Planning; CCWE</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S004896972205848X</t>
@@ -3796,7 +3795,7 @@
     <t xml:space="preserve">Larry.Engel@unc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("ExtraintestinalpathogenicE.coli(ExPEC)", "Foodborneurinarytractinfection(fUTI)", "Concentratedanimalfeedingoperation(CAFO)", "Syndromicsurveillance", "Besag-York-Mollié(BYM)model", "Ecologicalregressionanalysis")</t>
+    <t xml:space="preserve">ExtraintestinalpathogenicE.coli(ExPEC); Foodborneurinarytractinfection(fUTI); Concentratedanimalfeedingoperation(CAFO); Syndromicsurveillance; Besag-York-Mollié(BYM)model; Ecologicalregressionanalysis</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722059411</t>
@@ -3817,7 +3816,7 @@
     <t xml:space="preserve">djwallis@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Sourceapportionment", "Receptormodels", "PFAS", "Perfluoroalkylsubstances")</t>
+    <t xml:space="preserve">Sourceapportionment; Receptormodels; PFAS; Perfluoroalkylsubstances</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722054821</t>
@@ -3844,7 +3843,7 @@
     <t xml:space="preserve">Code can be found at the Github linked in the article: https://github.com/haleyplaas/CR-AS_2020/blob/v0.1/CR-AS%20data%20cleaning%2C%20stats%2C%20figures.R. Data can be made available upon request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Waterquality", "ToxicCyanobacteria", "Airquality", "PM2.5", "Microcystis", "Dolichospermum")</t>
+    <t xml:space="preserve">Waterquality; ToxicCyanobacteria; Airquality; PM2.5; Microcystis; Dolichospermum</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0376738822006019</t>
@@ -3874,7 +3873,7 @@
     <t xml:space="preserve">0000-0002-7018-391X</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Permeance", "Selectivity", "Rejection", "Advectivetransport", "Diffusivetransport")</t>
+    <t xml:space="preserve">Permeance; Selectivity; Rejection; Advectivetransport; Diffusivetransport</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0301479722009070</t>
@@ -3907,7 +3906,7 @@
     <t xml:space="preserve">0000-0003-3896-1483</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Nutrientmanagement", "Livestock", "Agriculture", "Machinelearning", "SatelliteradarSentinel-1")</t>
+    <t xml:space="preserve">Nutrientmanagement; Livestock; Agriculture; Machinelearning; SatelliteradarSentinel-1</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0272771422002311</t>
@@ -3937,7 +3936,7 @@
     <t xml:space="preserve">Data are available in supplemental tables. Code will be shared upon request.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Nitrogenremoval", "Denitrification", "Anammox", "nosZ", "hzo", "Sediments")</t>
+    <t xml:space="preserve">Nitrogenremoval; Denitrification; Anammox; nosZ; hzo; Sediments</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722019167</t>
@@ -3958,7 +3957,7 @@
     <t xml:space="preserve">arborqui@usc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("CAFOs", "Swine", "Hogproduction", "Animalfarming", "Environmentaljustice", "Gastrointestinalillness")</t>
+    <t xml:space="preserve">CAFOs; Swine; Hogproduction; Animalfarming; Environmentaljustice; Gastrointestinalillness</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722018563?via%3Dihub</t>
@@ -3970,7 +3969,7 @@
     <t xml:space="preserve">Department of Marine, Earth, and Atmospheric Sciences, North Carolina State University, Raleigh, NC, United States</t>
   </si>
   <si>
-    <t xml:space="preserve">c("PFAS", "Massload", "Model", "Sourcetracking", "Environmentalmonitoring", "Drinkingwater")</t>
+    <t xml:space="preserve">PFAS; Massload; Model; Sourcetracking; Environmentalmonitoring; Drinkingwater</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722022951?via%3Dihub</t>
@@ -3997,7 +3996,7 @@
     <t xml:space="preserve">aharris5@ncsu.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Animalhusbandry", "Fecalcontamination", "Sanitation", "Hygiene", "Animalfecesmanagement", "Entericpathogens")</t>
+    <t xml:space="preserve">Animalhusbandry; Fecalcontamination; Sanitation; Hygiene; Animalfecesmanagement; Entericpathogens</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0925857422001574</t>
@@ -4009,7 +4008,7 @@
     <t xml:space="preserve">Department of Biological and Agricultural Engineering, North Carolina State University, 3100 Faucette Dr., Raleigh, NC 27695, United States of America</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Naturalinfrastructure", "Wetlandrestoration", "Reforestation", "Watershedmodeling")</t>
+    <t xml:space="preserve">Naturalinfrastructure; Wetlandrestoration; Reforestation; Watershedmodeling</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S027843432200142X</t>
@@ -4030,7 +4029,7 @@
     <t xml:space="preserve">nfiori@umich.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Hydrogeology", "Climatechange", "Sea-levelrise", "Saltwaterintrusion", "Barrier-islandaquifers")</t>
+    <t xml:space="preserve">Hydrogeology; Climatechange; Sea-levelrise; Saltwaterintrusion; Barrier-islandaquifers</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0043135422007552</t>
@@ -4051,7 +4050,7 @@
     <t xml:space="preserve">0000-0003-1322-1948</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Advancedmeteringinfrastructure", "Waterserviceinterruption", "WaterUtilities", "Smartmeters")</t>
+    <t xml:space="preserve">Advancedmeteringinfrastructure; Waterserviceinterruption; WaterUtilities; Smartmeters</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0160412022001027</t>
@@ -4081,7 +4080,7 @@
     <t xml:space="preserve">argos@uic.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Arsenic", "Privatewells", "Watercontamination", "Birthoutcomes", "Epidemiology")</t>
+    <t xml:space="preserve">Arsenic; Privatewells; Watercontamination; Birthoutcomes; Epidemiology</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722002431</t>
@@ -4102,7 +4101,7 @@
     <t xml:space="preserve">yuezhi6170@163.com</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Lanthanumcontainingmaterial", "Lanthanumcarbonate", "Phosphorusremoval", "Wastewatertreatment", "Mineralprecipitation")</t>
+    <t xml:space="preserve">Lanthanumcontainingmaterial; Lanthanumcarbonate; Phosphorusremoval; Wastewatertreatment; Mineralprecipitation</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969722024949?via%3Dihub</t>
@@ -4126,7 +4125,7 @@
     <t xml:space="preserve">sonia.grego@duke.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Residencehall", "Asymptomaticsurveillance", "Positivepredictivevalue", "Clinicalcase")</t>
+    <t xml:space="preserve">Residencehall; Asymptomaticsurveillance; Positivepredictivevalue; Clinicalcase</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0301479722005771</t>
@@ -4153,7 +4152,7 @@
     <t xml:space="preserve">0000-0001-6020-9250</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Infiltrationcapacity", "Urbanhydrology", "Urbansoil", "Rainfall-runoffmodels", "Randomforest", "Stormwater")</t>
+    <t xml:space="preserve">Infiltrationcapacity; Urbanhydrology; Urbansoil; Rainfall-runoffmodels; Randomforest; Stormwater</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S2352801X22000364</t>
@@ -4183,7 +4182,7 @@
     <t xml:space="preserve">0000-0002-4606-9973</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Groundwater", "Microbesampling", "NorthCarolina", "Coliform", "E.coli", "Waterquality")</t>
+    <t xml:space="preserve">Groundwater; Microbesampling; NorthCarolina; Coliform; E.coli; Waterquality</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S2772411522000088</t>
@@ -4198,7 +4197,7 @@
     <t xml:space="preserve">Department of Forestry and Environmental Resources, North Carolina State University, Raleigh, N.C., U.SA.</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Rurallandscapes", "Nature-basedsolutions", "Costs", "Economics", "Capitalbudgeting", "Floodmitigation")</t>
+    <t xml:space="preserve">Rurallandscapes; Nature-basedsolutions; Costs; Economics; Capitalbudgeting; Floodmitigation</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S014362282200008X</t>
@@ -4222,7 +4221,7 @@
     <t xml:space="preserve">0000-0002-9380-7625</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Aquaticecosystems", "Hydrology", "Landuse/landcover", "Physicalhabitat", "Urbanstreams", "Waterquality")</t>
+    <t xml:space="preserve">Aquaticecosystems; Hydrology; Landuse/landcover; Physicalhabitat; Urbanstreams; Waterquality</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S0048969721075811</t>
@@ -4246,7 +4245,7 @@
     <t xml:space="preserve">mmunir@uncc.edu</t>
   </si>
   <si>
-    <t xml:space="preserve">c("SARS-CoV-2", "Wastewater", "COVID-19", "RT-qPCR", "RT-ddPCR", "Wastewater-basedepidemiology(WBE)")</t>
+    <t xml:space="preserve">SARS-CoV-2; Wastewater; COVID-19; RT-qPCR; RT-ddPCR; Wastewater-basedepidemiology(WBE)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0378377422001391</t>
@@ -4261,7 +4260,7 @@
     <t xml:space="preserve">Department of Biological and Agricultural Engineering, North Carolina State University, Weaver Laboratory, 3110 Faucette Dr., Raleigh, NC 27695-7625, USA</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Subsurfacedrainage", "Supplementalirrigation", "On-farmwaterstorage", "Irrigationreservoir", "Drainagewaterreuse", "DRAINMOD-DWR")</t>
+    <t xml:space="preserve">Subsurfacedrainage; Supplementalirrigation; On-farmwaterstorage; Irrigationreservoir; Drainagewaterreuse; DRAINMOD-DWR</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969722019167?via%3Dihub</t>
@@ -4276,7 +4275,7 @@
     <t xml:space="preserve">https://ars.els-cdn.com/content/image/1-s2.0-S0048969721065578-mmc1.docx</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Arsenic", "Manganese", "Lead", "Privatewells", "K-meansclustering", "Geocoding")</t>
+    <t xml:space="preserve">Arsenic; Manganese; Lead; Privatewells; K-meansclustering; Geocoding</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/abs/pii/S0048969721061866</t>
@@ -4288,7 +4287,7 @@
     <t xml:space="preserve">https://ars.els-cdn.com/content/image/1-s2.0-S0048969721061866-mmc1.docx</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Floods", "Hurricanes", "Interruptedtimeseriesanalysis", "Gastrointestinalillness", "Environmentalepidemiology", "Disasterepidemiology")</t>
+    <t xml:space="preserve">Floods; Hurricanes; Interruptedtimeseriesanalysis; Gastrointestinalillness; Environmentalepidemiology; Disasterepidemiology</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S001393512101447X</t>
@@ -4309,7 +4308,7 @@
     <t xml:space="preserve">Department of Environmental Sciences and Engineering, Gillings School of Global Public Health, University of North Carolina at Chapel Hill, 135 Dauer Drive, Chapel Hill, NC, 27599, USA</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Bayesiannetworks", "Drinkingwater", "Bloodleadlevels", "Machinelearning", "Riskassessment", "Healthdisparity")</t>
+    <t xml:space="preserve">Bayesiannetworks; Drinkingwater; Bloodleadlevels; Machinelearning; Riskassessment; Healthdisparity</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.sciencedirect.com/science/article/pii/S004896972105525X</t>
@@ -4324,7 +4323,7 @@
     <t xml:space="preserve">University of North Carolina at Chapel Hill, Gillings School of Global Public Health, Department of Environmental Science &amp; Engineering, 135 Dauer Drive, Chapel Hill, NC 27599, United States of America</t>
   </si>
   <si>
-    <t xml:space="preserve">c("Privatewells", "Householdwatertreatment", "Healthbeliefmodel", "Self-efficacy", "Socialcognitivetheory", "Drinkingwater")</t>
+    <t xml:space="preserve">Privatewells; Householdwatertreatment; Healthbeliefmodel; Self-efficacy; Socialcognitivetheory; Drinkingwater</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Rewrite expired supp_url and paper_url links to stable locations (#10)
343 washdev supp_url values were pre-signed Silverchair CDN links that
expired in January 2024, and 3 uncnewsletter paper_url values were Google
Scholar alert redirects. Both are now canonical: the Silverchair links
become https://doi.org/<doi> URLs (the DOI is recovered from the link
path), and the Scholar redirects are decoded to their target URLs. The
high-entropy Signature and scisig tokens that tripped secret scanners are
gone. No re-collection was needed.

Two reproducible helpers in data-raw/helpers.R do the rewrites:
canonicalize_silverchair_url() and decode_scholar_redirect(). Only
washdev$supp_url and uncnewsletter$paper_url changed; row counts and all
other columns are identical, and ploswater is untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/uncnewsletter.xlsx
+++ b/inst/extdata/uncnewsletter.xlsx
@@ -1535,7 +1535,7 @@
     <t xml:space="preserve">biology-geologyfeebacks; DMQ99; evapotranspiration; headwaterstreams; landusechange; seasonalflashiness; specificconductance; streamgauges</t>
   </si>
   <si>
-    <t xml:space="preserve">https://scholar.google.com/scholar_url?url=https://ajph.aphapublications.org/doi/pdf/10.2105/AJPH.2022.307003%3Fdownload%3Dtrue&amp;hl=en&amp;sa=X&amp;d=3962241131938486649&amp;ei=H1Q7Y6aFPO2KywSS3bH4Bg&amp;scisig=AAGBfm3Q4X2sCbJJGTgTcSrsGU_FdUVJcw&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:7463423130094204642:AAGBfm306n8jEm7p9E06Y9mqflGSBiV6Pg&amp;html=&amp;pos=0&amp;folt=kw-top</t>
+    <t xml:space="preserve">https://ajph.aphapublications.org/doi/pdf/10.2105/AJPH.2022.307003?download=true</t>
   </si>
   <si>
     <t xml:space="preserve">scholar.google.com</t>
@@ -1559,7 +1559,7 @@
     <t xml:space="preserve">0000-0003-3641-737X</t>
   </si>
   <si>
-    <t xml:space="preserve">https://scholar.google.com/scholar_url?url=https://pubs.acs.org/doi/full/10.1021/acsestwater.2c00157&amp;hl=en&amp;sa=X&amp;d=1709742523088559831&amp;ei=Dg_7YtkJhJjLBKCbvNAC&amp;scisig=AAGBfm0jov0_aWmZMwe4s6j4e9vubbdcbA&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:3226461804228696973:AAGBfm3ju-C3kL6mSiPesevK78XQ69Qd6A&amp;html=&amp;pos=2&amp;folt=kw</t>
+    <t xml:space="preserve">https://pubs.acs.org/doi/full/10.1021/acsestwater.2c00157</t>
   </si>
   <si>
     <t xml:space="preserve">ACS EST Water</t>
@@ -1586,7 +1586,7 @@
     <t xml:space="preserve">WASP; environmentalmodeling; nanocopper; nanomaterials; freswater</t>
   </si>
   <si>
-    <t xml:space="preserve">https://scholar.google.com/scholar_url?url=https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/hir.12445&amp;hl=en&amp;sa=X&amp;d=7293212103073901469&amp;ei=2fm2YrzQKtHjmQGNwb84&amp;scisig=AAGBfm1zjx3-V2aCgS0L1xZx26MYDvF-tg&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:3552202248086981277:AAGBfm3xoOKMdpREzJ__fgBb7pdlMpLHFA&amp;html=&amp;pos=1&amp;folt=kw</t>
+    <t xml:space="preserve">https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/hir.12445</t>
   </si>
   <si>
     <t xml:space="preserve">Health Information and Libraries Journal</t>

</xml_diff>